<commit_message>
🐛🎮 Corrige configuración de cantidades y objetivos del portal de juegos
🐛 Corregido el campo Juegos requeridos para completar que regresaba incorrectamente al valor máximo
🔢 Permitido ingresar libremente cantidades entre 1 y el máximo de juegos disponibles
🎮 Corregido el mismo comportamiento en Cantidad de juegos
⌨️ El valor actual se selecciona al enfocar el campo para facilitar su reemplazo
⚡ El resumen de reglas continúa actualizándose en tiempo real sin modificar lo que el usuario está escribiendo
✅ Los valores se normalizan únicamente al salir del campo, cambiar la configuración o guardar
🛡️ Se mantiene la validación del backend para impedir cantidades superiores a los juegos realmente disponibles
🧹 Mejorada la consistencia y experiencia de configuración del portal de juegos
</commit_message>
<xml_diff>
--- a/plantilla_empleados.xlsx
+++ b/plantilla_empleados.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empleados" sheetId="1" r:id="Rfdb3def80b9e41f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rf0dadc7ad88c405a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empleados" sheetId="1" r:id="Ra5e6f4d6ac4c4cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R71e8ad85316047c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -118,6 +118,7 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -324,6 +325,7 @@
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -338,6 +340,9 @@
       </x:c>
       <x:c r="D1" s="5" t="str">
         <x:v>Correo</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Estado</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="20" customHeight="1">
@@ -1597,11 +1602,21 @@
         <x:v>Opcional. Si se completa, debe ser un correo válido.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" t="str">
+        <x:v>Estado</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Opcional. Usa Activo o Inactivo. Si se deja vacío, se importa como Activo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="26" t="str">
-        <x:v>Importante: no agregues una columna Estado. Los empleados nuevos se importan como activos por defecto.</x:v>
-      </x:c>
-      <x:c r="B9" s="26"/>
+        <x:v>Compatibilidad</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="str">
+        <x:v>La plantilla y los archivos exportados pueden volver a importarse; las columnas adicionales de exportación se ignoran cuando no son necesarias.</x:v>
+      </x:c>
       <x:c r="C9" s="26"/>
       <x:c r="D9" s="26"/>
       <x:c r="E9" s="26"/>

</xml_diff>